<commit_message>
Checkpoint after real Excel migration
</commit_message>
<xml_diff>
--- a/سیستم انبار.xlsx
+++ b/سیستم انبار.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Work\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78E3893C-24BD-4535-9269-177DEE3E11A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43F02CF6-7F6B-4115-B2C9-548F8E0F8D89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13140" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13140" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="کالاها" sheetId="6" r:id="rId1"/>
@@ -70,7 +70,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="434" uniqueCount="154">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="422" uniqueCount="146">
   <si>
     <t>ردیف</t>
   </si>
@@ -492,34 +492,10 @@
     <t>مانده</t>
   </si>
   <si>
-    <t>R-050617-174</t>
-  </si>
-  <si>
-    <t>R-050617-176</t>
-  </si>
-  <si>
-    <t>R-050617-177</t>
-  </si>
-  <si>
-    <t>R-050617-178</t>
-  </si>
-  <si>
     <t>1405/06/18</t>
   </si>
   <si>
     <t>1405/06/19</t>
-  </si>
-  <si>
-    <t>1405/06/20</t>
-  </si>
-  <si>
-    <t>1405/06/21</t>
-  </si>
-  <si>
-    <t>1405/06/22</t>
-  </si>
-  <si>
-    <t>تستی</t>
   </si>
   <si>
     <t>H-050617-2</t>
@@ -914,7 +890,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="74">
+  <cellXfs count="70">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1002,127 +978,117 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1293,30 +1259,6 @@
         <top/>
         <bottom/>
       </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -1576,6 +1518,30 @@
         </horizontal>
       </border>
     </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -1590,59 +1556,59 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{279CBFD2-2AC2-433F-9662-32BD9036D34C}" name="tblkala" displayName="tblkala" ref="A1:G29" totalsRowShown="0" headerRowDxfId="39" dataDxfId="37" headerRowBorderDxfId="38" tableBorderDxfId="36" totalsRowBorderDxfId="35">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{279CBFD2-2AC2-433F-9662-32BD9036D34C}" name="tblkala" displayName="tblkala" ref="A1:G29" totalsRowShown="0" headerRowDxfId="31" dataDxfId="29" headerRowBorderDxfId="30" tableBorderDxfId="28" totalsRowBorderDxfId="27">
   <autoFilter ref="A1:G29" xr:uid="{279CBFD2-2AC2-433F-9662-32BD9036D34C}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{148E244A-7F43-42C6-9787-E5D8735C5902}" name="کد  کالا" dataDxfId="34"/>
-    <tableColumn id="2" xr3:uid="{43E86D7D-9E75-47C4-9F50-3811296F5D01}" name="عنوان کالا" dataDxfId="33"/>
-    <tableColumn id="3" xr3:uid="{5A5F8A33-8AAC-4B49-AD51-0219D1549F82}" name="گروه" dataDxfId="32"/>
-    <tableColumn id="4" xr3:uid="{68A6FE96-BB6C-47CE-BAF3-A4CFC1C7070E}" name="زیرگروه" dataDxfId="31"/>
-    <tableColumn id="5" xr3:uid="{0E7081B2-3B76-455F-97B7-FE57F5B24AD2}" name="واحد" dataDxfId="30"/>
-    <tableColumn id="6" xr3:uid="{D1166D98-ACD6-41F8-A7BC-9F140BE67088}" name="حداقل موجودی" dataDxfId="29"/>
-    <tableColumn id="7" xr3:uid="{C601BDE2-F9B9-42D1-B12D-B95A9AD1B607}" name="توضیحات" dataDxfId="28"/>
+    <tableColumn id="1" xr3:uid="{148E244A-7F43-42C6-9787-E5D8735C5902}" name="کد  کالا" dataDxfId="26"/>
+    <tableColumn id="2" xr3:uid="{43E86D7D-9E75-47C4-9F50-3811296F5D01}" name="عنوان کالا" dataDxfId="25"/>
+    <tableColumn id="3" xr3:uid="{5A5F8A33-8AAC-4B49-AD51-0219D1549F82}" name="گروه" dataDxfId="24"/>
+    <tableColumn id="4" xr3:uid="{68A6FE96-BB6C-47CE-BAF3-A4CFC1C7070E}" name="زیرگروه" dataDxfId="23"/>
+    <tableColumn id="5" xr3:uid="{0E7081B2-3B76-455F-97B7-FE57F5B24AD2}" name="واحد" dataDxfId="22"/>
+    <tableColumn id="6" xr3:uid="{D1166D98-ACD6-41F8-A7BC-9F140BE67088}" name="حداقل موجودی" dataDxfId="21"/>
+    <tableColumn id="7" xr3:uid="{C601BDE2-F9B9-42D1-B12D-B95A9AD1B607}" name="توضیحات" dataDxfId="20"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{646114BF-3D58-4F0A-9D7F-7D063CBCEC71}" name="tblvorood" displayName="tblvorood" ref="A1:H7" totalsRowShown="0" headerRowDxfId="27">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{646114BF-3D58-4F0A-9D7F-7D063CBCEC71}" name="tblvorood" displayName="tblvorood" ref="A1:H7" totalsRowShown="0" headerRowDxfId="19">
   <autoFilter ref="A1:H7" xr:uid="{646114BF-3D58-4F0A-9D7F-7D063CBCEC71}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{627C171E-63BF-4A3C-90DE-4CFC28D0D1CD}" name="شماره رسید" dataDxfId="26"/>
-    <tableColumn id="2" xr3:uid="{677D1096-D899-40E3-B1F6-04997B3AF8E1}" name="تاریخ" dataDxfId="25"/>
-    <tableColumn id="3" xr3:uid="{EA071B89-B617-4FCF-B459-896469F0AB8B}" name="ردیف" dataDxfId="24"/>
-    <tableColumn id="4" xr3:uid="{A022E81B-C7F4-4327-9277-8BFAFB1F7BFC}" name="کد کالا" dataDxfId="23"/>
-    <tableColumn id="5" xr3:uid="{4B5C5F2B-6172-4B80-AB31-3DEA5CD33B4D}" name="عنوان کالا" dataDxfId="22">
+    <tableColumn id="1" xr3:uid="{627C171E-63BF-4A3C-90DE-4CFC28D0D1CD}" name="شماره رسید" dataDxfId="18"/>
+    <tableColumn id="2" xr3:uid="{677D1096-D899-40E3-B1F6-04997B3AF8E1}" name="تاریخ" dataDxfId="17"/>
+    <tableColumn id="3" xr3:uid="{EA071B89-B617-4FCF-B459-896469F0AB8B}" name="ردیف" dataDxfId="16"/>
+    <tableColumn id="4" xr3:uid="{A022E81B-C7F4-4327-9277-8BFAFB1F7BFC}" name="کد کالا" dataDxfId="15"/>
+    <tableColumn id="5" xr3:uid="{4B5C5F2B-6172-4B80-AB31-3DEA5CD33B4D}" name="عنوان کالا" dataDxfId="14">
       <calculatedColumnFormula>IFERROR(_xlfn.XLOOKUP(D2,tblkala[کد  کالا],tblkala[عنوان کالا],""),"")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{C9CE9F8C-BB2E-40B8-A6C4-DBB58472EA6E}" name="مقدار" dataDxfId="21"/>
-    <tableColumn id="7" xr3:uid="{937AFE89-5466-44C3-B59E-DA55912441FE}" name="واحد" dataDxfId="20">
+    <tableColumn id="6" xr3:uid="{C9CE9F8C-BB2E-40B8-A6C4-DBB58472EA6E}" name="مقدار" dataDxfId="13"/>
+    <tableColumn id="7" xr3:uid="{937AFE89-5466-44C3-B59E-DA55912441FE}" name="واحد" dataDxfId="12">
       <calculatedColumnFormula>IFERROR(_xlfn.XLOOKUP(D2,tblkala[کد  کالا],tblkala[واحد],""),"")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{306C5378-106D-47E4-B61C-92C4CB871D65}" name="توضیحات" dataDxfId="19"/>
+    <tableColumn id="8" xr3:uid="{306C5378-106D-47E4-B61C-92C4CB871D65}" name="توضیحات" dataDxfId="11"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{32B5F06D-1838-4241-9D83-054BE1C79FD2}" name="tblkhorooj" displayName="tblkhorooj" ref="A1:J6" totalsRowShown="0" headerRowDxfId="18">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{32B5F06D-1838-4241-9D83-054BE1C79FD2}" name="tblkhorooj" displayName="tblkhorooj" ref="A1:J6" totalsRowShown="0" headerRowDxfId="39">
   <autoFilter ref="A1:J6" xr:uid="{32B5F06D-1838-4241-9D83-054BE1C79FD2}"/>
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{547F3829-8E7E-4239-B7F5-B439C80216AD}" name="شماره حواله" dataDxfId="17"/>
+    <tableColumn id="1" xr3:uid="{547F3829-8E7E-4239-B7F5-B439C80216AD}" name="شماره حواله" dataDxfId="38"/>
     <tableColumn id="2" xr3:uid="{17F4008B-1079-47E2-BF0D-7819E296486F}" name="تاریخ"/>
-    <tableColumn id="3" xr3:uid="{0DA6E170-3670-446C-B238-78F930466C1D}" name="ردیف" dataDxfId="16"/>
+    <tableColumn id="3" xr3:uid="{0DA6E170-3670-446C-B238-78F930466C1D}" name="ردیف" dataDxfId="37"/>
     <tableColumn id="4" xr3:uid="{B063A55B-A15E-4487-9A02-CB1FF0CC4A19}" name="کد کالا"/>
-    <tableColumn id="5" xr3:uid="{E5B24D1C-3166-4658-B852-B6BE009CD214}" name="عنوان کالا" dataDxfId="15">
+    <tableColumn id="5" xr3:uid="{E5B24D1C-3166-4658-B852-B6BE009CD214}" name="عنوان کالا" dataDxfId="36">
       <calculatedColumnFormula>IFERROR(_xlfn.XLOOKUP(D2,tblkala[کد  کالا],tblkala[عنوان کالا],""),"")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{D1CF82D4-73B1-4126-A389-9C9E1F8F8A57}" name="مقدار" dataDxfId="14"/>
-    <tableColumn id="7" xr3:uid="{15EB6DFF-B6B0-4563-9490-EB434404C9E6}" name="واحد" dataDxfId="13">
+    <tableColumn id="6" xr3:uid="{D1CF82D4-73B1-4126-A389-9C9E1F8F8A57}" name="مقدار" dataDxfId="35"/>
+    <tableColumn id="7" xr3:uid="{15EB6DFF-B6B0-4563-9490-EB434404C9E6}" name="واحد" dataDxfId="34">
       <calculatedColumnFormula>IFERROR(_xlfn.XLOOKUP(D2,tblkala[کد  کالا],tblkala[واحد],""),"")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{43C3D014-A3CA-484E-8FB9-23397CB6BEF7}" name="تحویل گیرنده" dataDxfId="12"/>
-    <tableColumn id="9" xr3:uid="{DC81FA74-BD76-4EFE-93FB-B684DBA4E31E}" name="محل مصرف" dataDxfId="11"/>
+    <tableColumn id="8" xr3:uid="{43C3D014-A3CA-484E-8FB9-23397CB6BEF7}" name="تحویل گیرنده" dataDxfId="33"/>
+    <tableColumn id="9" xr3:uid="{DC81FA74-BD76-4EFE-93FB-B684DBA4E31E}" name="محل مصرف" dataDxfId="32"/>
     <tableColumn id="10" xr3:uid="{CBA0F31D-9D38-436D-9480-8AF31ACAE0DC}" name="توضیحات"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -2610,95 +2576,23 @@
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
-        <v>140</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>144</v>
-      </c>
-      <c r="C4" s="2">
-        <v>3</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="E4" s="2" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(D4,tblkala[کد  کالا],tblkala[عنوان کالا],""),"")</f>
-        <v>پیچ پنل 25 میلی TN25</v>
-      </c>
-      <c r="F4" s="1">
-        <v>10</v>
-      </c>
-      <c r="G4" s="1" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(D4,tblkala[کد  کالا],tblkala[واحد],""),"")</f>
-        <v>بسته</v>
-      </c>
-      <c r="H4" s="2" t="s">
-        <v>149</v>
-      </c>
+      <c r="C4" s="2"/>
+      <c r="E4" s="2"/>
+      <c r="H4" s="2"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
-        <v>141</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="C5" s="2">
-        <v>4</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="E5" s="2" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(D5,tblkala[کد  کالا],tblkala[عنوان کالا],""),"")</f>
-        <v>پیچ پنل 25 میلی TN25</v>
-      </c>
-      <c r="F5" s="1">
-        <v>7</v>
-      </c>
-      <c r="G5" s="1" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(D5,tblkala[کد  کالا],tblkala[واحد],""),"")</f>
-        <v>بسته</v>
-      </c>
-      <c r="H5" s="2" t="s">
-        <v>152</v>
-      </c>
+      <c r="C5" s="2"/>
+      <c r="E5" s="2"/>
+      <c r="H5" s="2"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>147</v>
-      </c>
       <c r="C6" s="2"/>
-      <c r="E6" s="2" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(D6,tblkala[کد  کالا],tblkala[عنوان کالا],""),"")</f>
-        <v/>
-      </c>
-      <c r="G6" s="1" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(D6,tblkala[کد  کالا],tblkala[واحد],""),"")</f>
-        <v/>
-      </c>
+      <c r="E6" s="2"/>
       <c r="H6" s="2"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
-        <v>143</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>148</v>
-      </c>
       <c r="C7" s="2"/>
-      <c r="E7" s="2" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(D7,tblkala[کد  کالا],tblkala[عنوان کالا],""),"")</f>
-        <v/>
-      </c>
-      <c r="G7" s="1" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(D7,tblkala[کد  کالا],tblkala[واحد],""),"")</f>
-        <v/>
-      </c>
+      <c r="E7" s="2"/>
       <c r="H7" s="2"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -2846,10 +2740,10 @@
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>150</v>
+        <v>142</v>
       </c>
       <c r="B3" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="C3" s="1">
         <v>2</v>
@@ -2869,21 +2763,21 @@
         <v>بسته</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>151</v>
+        <v>143</v>
       </c>
       <c r="I3" s="1" t="s">
         <v>137</v>
       </c>
       <c r="J3" t="s">
-        <v>152</v>
+        <v>144</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>153</v>
+        <v>145</v>
       </c>
       <c r="B4" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="C4" s="1">
         <v>3</v>
@@ -2903,13 +2797,13 @@
         <v>بسته</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>151</v>
+        <v>143</v>
       </c>
       <c r="I4" s="1" t="s">
         <v>137</v>
       </c>
       <c r="J4" t="s">
-        <v>152</v>
+        <v>144</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
@@ -3389,7 +3283,7 @@
       </c>
       <c r="F11" s="2">
         <f>SUMIF(tblvorood[کد کالا],A11,tblvorood[مقدار])</f>
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="G11" s="2">
         <f>SUMIF(tblkhorooj[کد کالا],A11,tblkhorooj[مقدار])</f>
@@ -3397,7 +3291,7 @@
       </c>
       <c r="H11" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A11,tblMabna[کد کالا],tblMabna[مقدار مبنا],0)+F11-G11,0)</f>
-        <v>44</v>
+        <v>27</v>
       </c>
       <c r="I11" s="2">
         <f>IFERROR(_xlfn.XLOOKUP(A11,tblkala[کد  کالا],tblkala[حداقل موجودی],""),"")</f>
@@ -4167,45 +4061,45 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="39" t="s">
+      <c r="A1" s="49" t="s">
         <v>19</v>
       </c>
-      <c r="B1" s="40"/>
-      <c r="C1" s="40"/>
-      <c r="D1" s="40"/>
-      <c r="E1" s="40"/>
+      <c r="B1" s="50"/>
+      <c r="C1" s="50"/>
+      <c r="D1" s="50"/>
+      <c r="E1" s="50"/>
     </row>
     <row r="2" spans="1:5" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="41" t="s">
+      <c r="A2" s="51" t="s">
         <v>20</v>
       </c>
-      <c r="B2" s="41"/>
-      <c r="C2" s="41"/>
-      <c r="D2" s="41"/>
-      <c r="E2" s="41"/>
+      <c r="B2" s="51"/>
+      <c r="C2" s="51"/>
+      <c r="D2" s="51"/>
+      <c r="E2" s="51"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="42" t="s">
+      <c r="A3" s="48" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="42"/>
-      <c r="C3" s="44" t="s">
+      <c r="B3" s="48"/>
+      <c r="C3" s="52" t="s">
         <v>130</v>
       </c>
-      <c r="D3" s="44"/>
-      <c r="E3" s="44"/>
+      <c r="D3" s="52"/>
+      <c r="E3" s="52"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="42" t="s">
+      <c r="A4" s="48" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="42"/>
-      <c r="C4" s="42" t="str">
+      <c r="B4" s="48"/>
+      <c r="C4" s="48" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(C3,tblvorood[شماره رسید],tblvorood[تاریخ],""),"")</f>
         <v>1405/06/17</v>
       </c>
-      <c r="D4" s="42"/>
-      <c r="E4" s="42"/>
+      <c r="D4" s="48"/>
+      <c r="E4" s="48"/>
     </row>
     <row r="6" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
@@ -4225,138 +4119,137 @@
       </c>
     </row>
     <row r="7" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="72" cm="1">
+      <c r="A7" s="47" cm="1">
         <f t="array" ref="A7:A8">_xlfn._xlws.FILTER(tblvorood[ردیف],tblvorood[شماره رسید]=C3,"")</f>
         <v>1</v>
       </c>
-      <c r="B7" s="72" t="str" cm="1">
+      <c r="B7" s="47" t="str" cm="1">
         <f t="array" ref="B7:B8">_xlfn._xlws.FILTER(tblvorood[عنوان کالا],tblvorood[شماره رسید]=C3,"")</f>
         <v>استاد C 100*3500</v>
       </c>
-      <c r="C7" s="72" cm="1">
+      <c r="C7" s="47" cm="1">
         <f t="array" ref="C7:C8">_xlfn._xlws.FILTER(tblvorood[مقدار],tblvorood[شماره رسید]=C3,"")</f>
         <v>300</v>
       </c>
-      <c r="D7" s="72" t="str" cm="1">
+      <c r="D7" s="47" t="str" cm="1">
         <f t="array" ref="D7:D8">_xlfn._xlws.FILTER(tblvorood[واحد],tblvorood[شماره رسید]=C3,"")</f>
         <v>شاخه</v>
       </c>
-      <c r="E7" s="72" t="str" cm="1">
+      <c r="E7" s="47" t="str" cm="1">
         <f t="array" ref="E7:E8">_xlfn._xlws.FILTER(tblvorood[توضیحات],tblvorood[شماره رسید]=C3,"")</f>
         <v>برگ خروج انبار 3539 (1050 متر طول)</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="72">
+      <c r="A8" s="47">
         <v>2</v>
       </c>
-      <c r="B8" s="72" t="str">
+      <c r="B8" s="47" t="str">
         <v>استاد C 100*3500</v>
       </c>
-      <c r="C8" s="72">
+      <c r="C8" s="47">
         <v>750</v>
       </c>
-      <c r="D8" s="72" t="str">
+      <c r="D8" s="47" t="str">
         <v>شاخه</v>
       </c>
-      <c r="E8" s="72" t="str">
+      <c r="E8" s="47" t="str">
         <v>برگ خروج انبار 3540 (2625 متر طول)</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="72"/>
-      <c r="B9" s="72"/>
-      <c r="C9" s="72"/>
-      <c r="D9" s="72"/>
-      <c r="E9" s="72"/>
+      <c r="A9" s="47"/>
+      <c r="B9" s="47"/>
+      <c r="C9" s="47"/>
+      <c r="D9" s="47"/>
+      <c r="E9" s="47"/>
     </row>
     <row r="10" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="72"/>
-      <c r="B10" s="72"/>
-      <c r="C10" s="72"/>
-      <c r="D10" s="72"/>
-      <c r="E10" s="72"/>
+      <c r="A10" s="47"/>
+      <c r="B10" s="47"/>
+      <c r="C10" s="47"/>
+      <c r="D10" s="47"/>
+      <c r="E10" s="47"/>
     </row>
     <row r="11" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="72"/>
-      <c r="B11" s="72"/>
-      <c r="C11" s="72"/>
-      <c r="D11" s="72"/>
-      <c r="E11" s="72"/>
+      <c r="A11" s="47"/>
+      <c r="B11" s="47"/>
+      <c r="C11" s="47"/>
+      <c r="D11" s="47"/>
+      <c r="E11" s="47"/>
     </row>
     <row r="12" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="72"/>
-      <c r="B12" s="72"/>
-      <c r="C12" s="72"/>
-      <c r="D12" s="72"/>
-      <c r="E12" s="72"/>
+      <c r="A12" s="47"/>
+      <c r="B12" s="47"/>
+      <c r="C12" s="47"/>
+      <c r="D12" s="47"/>
+      <c r="E12" s="47"/>
     </row>
     <row r="13" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="72"/>
-      <c r="B13" s="72"/>
-      <c r="C13" s="72"/>
-      <c r="D13" s="72"/>
-      <c r="E13" s="72"/>
+      <c r="A13" s="47"/>
+      <c r="B13" s="47"/>
+      <c r="C13" s="47"/>
+      <c r="D13" s="47"/>
+      <c r="E13" s="47"/>
     </row>
     <row r="14" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="72"/>
-      <c r="B14" s="72"/>
-      <c r="C14" s="72"/>
-      <c r="D14" s="72"/>
-      <c r="E14" s="72"/>
+      <c r="A14" s="47"/>
+      <c r="B14" s="47"/>
+      <c r="C14" s="47"/>
+      <c r="D14" s="47"/>
+      <c r="E14" s="47"/>
     </row>
     <row r="15" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="72"/>
-      <c r="B15" s="72"/>
-      <c r="C15" s="72"/>
-      <c r="D15" s="72"/>
-      <c r="E15" s="72"/>
+      <c r="A15" s="47"/>
+      <c r="B15" s="47"/>
+      <c r="C15" s="47"/>
+      <c r="D15" s="47"/>
+      <c r="E15" s="47"/>
     </row>
     <row r="16" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="72"/>
-      <c r="B16" s="72"/>
-      <c r="C16" s="72"/>
-      <c r="D16" s="72"/>
-      <c r="E16" s="72"/>
+      <c r="A16" s="47"/>
+      <c r="B16" s="47"/>
+      <c r="C16" s="47"/>
+      <c r="D16" s="47"/>
+      <c r="E16" s="47"/>
     </row>
     <row r="17" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="72"/>
-      <c r="B17" s="72"/>
-      <c r="C17" s="72"/>
-      <c r="D17" s="72"/>
-      <c r="E17" s="72"/>
+      <c r="A17" s="47"/>
+      <c r="B17" s="47"/>
+      <c r="C17" s="47"/>
+      <c r="D17" s="47"/>
+      <c r="E17" s="47"/>
     </row>
     <row r="18" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="72"/>
-      <c r="B18" s="72"/>
-      <c r="C18" s="72"/>
-      <c r="D18" s="72"/>
-      <c r="E18" s="72"/>
+      <c r="A18" s="47"/>
+      <c r="B18" s="47"/>
+      <c r="C18" s="47"/>
+      <c r="D18" s="47"/>
+      <c r="E18" s="47"/>
     </row>
     <row r="19" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="72"/>
-      <c r="B19" s="72"/>
-      <c r="C19" s="72"/>
-      <c r="D19" s="72"/>
-      <c r="E19" s="72"/>
+      <c r="A19" s="47"/>
+      <c r="B19" s="47"/>
+      <c r="C19" s="47"/>
+      <c r="D19" s="47"/>
+      <c r="E19" s="47"/>
     </row>
     <row r="20" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="72"/>
-      <c r="B20" s="72"/>
-      <c r="C20" s="72"/>
-      <c r="D20" s="72"/>
-      <c r="E20" s="72"/>
+      <c r="A20" s="47"/>
+      <c r="B20" s="47"/>
+      <c r="C20" s="47"/>
+      <c r="D20" s="47"/>
+      <c r="E20" s="47"/>
     </row>
     <row r="21" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A22" s="73"/>
       <c r="B22" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="C22" s="42" t="s">
+      <c r="C22" s="48" t="s">
         <v>22</v>
       </c>
-      <c r="D22" s="42"/>
+      <c r="D22" s="48"/>
       <c r="E22" t="s">
         <v>23</v>
       </c>
@@ -4413,53 +4306,53 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A1" s="39" t="s">
+      <c r="A1" s="49" t="s">
         <v>19</v>
       </c>
-      <c r="B1" s="39"/>
-      <c r="C1" s="39"/>
-      <c r="D1" s="39"/>
-      <c r="E1" s="39"/>
-      <c r="F1" s="39"/>
+      <c r="B1" s="49"/>
+      <c r="C1" s="49"/>
+      <c r="D1" s="49"/>
+      <c r="E1" s="49"/>
+      <c r="F1" s="49"/>
     </row>
     <row r="2" spans="1:6" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="41" t="s">
+      <c r="A2" s="51" t="s">
         <v>26</v>
       </c>
-      <c r="B2" s="41"/>
-      <c r="C2" s="41"/>
-      <c r="D2" s="41"/>
-      <c r="E2" s="41"/>
-      <c r="F2" s="41"/>
-    </row>
-    <row r="3" spans="1:6" s="49" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="68" t="s">
+      <c r="B2" s="51"/>
+      <c r="C2" s="51"/>
+      <c r="D2" s="51"/>
+      <c r="E2" s="51"/>
+      <c r="F2" s="51"/>
+    </row>
+    <row r="3" spans="1:6" s="35" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="55" t="s">
         <v>13</v>
       </c>
-      <c r="B3" s="68"/>
-      <c r="C3" s="45" t="s">
-        <v>153</v>
-      </c>
-      <c r="D3" s="45"/>
-      <c r="E3" s="45"/>
+      <c r="B3" s="55"/>
+      <c r="C3" s="56" t="s">
+        <v>145</v>
+      </c>
+      <c r="D3" s="56"/>
+      <c r="E3" s="56"/>
     </row>
     <row r="4" spans="1:6" s="16" customFormat="1" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="43" t="s">
+      <c r="A4" s="57" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="43"/>
-      <c r="C4" s="43" t="str">
+      <c r="B4" s="57"/>
+      <c r="C4" s="57" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(C3,tblkhorooj[شماره حواله],tblkhorooj[تاریخ],""),"")</f>
         <v>1405/06/19</v>
       </c>
-      <c r="D4" s="43"/>
-      <c r="E4" s="43"/>
+      <c r="D4" s="57"/>
+      <c r="E4" s="57"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="69" t="s">
+      <c r="A5" s="53" t="s">
         <v>14</v>
       </c>
-      <c r="B5" s="70"/>
+      <c r="B5" s="54"/>
       <c r="C5" s="17" t="str">
         <f>IFERROR(_xlfn.XLOOKUP($C$3,tblkhorooj[شماره حواله],tblkhorooj[تحویل گیرنده],""),"")</f>
         <v>تیم قهرمانی</v>
@@ -4467,11 +4360,11 @@
       <c r="D5" s="9" t="s">
         <v>106</v>
       </c>
-      <c r="E5" s="70" t="str">
+      <c r="E5" s="54" t="str">
         <f>IFERROR(_xlfn.XLOOKUP($C$3,tblkhorooj[شماره حواله],tblkhorooj[محل مصرف],""),"")</f>
         <v>طبقه اول</v>
       </c>
-      <c r="F5" s="71"/>
+      <c r="F5" s="58"/>
     </row>
     <row r="7" spans="1:6" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
@@ -4493,130 +4386,130 @@
         <v>7</v>
       </c>
     </row>
-    <row r="8" spans="1:6" s="50" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="72" cm="1">
+    <row r="8" spans="1:6" s="36" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="47" cm="1">
         <f t="array" ref="A8:F8">IFERROR(_xlfn._xlws.FILTER(_xlfn.CHOOSECOLS(tblkhorooj[],3,4,5,6,7,10),tblkhorooj[شماره حواله]=$C$3),"")</f>
         <v>3</v>
       </c>
-      <c r="B8" s="72" t="str">
+      <c r="B8" s="47" t="str">
         <v>K010</v>
       </c>
-      <c r="C8" s="72" t="str">
+      <c r="C8" s="47" t="str">
         <v>پیچ پنل 25 میلی TN25</v>
       </c>
-      <c r="D8" s="72">
+      <c r="D8" s="47">
         <v>12</v>
       </c>
-      <c r="E8" s="72" t="str">
+      <c r="E8" s="47" t="str">
         <v>بسته</v>
       </c>
-      <c r="F8" s="72" t="str">
+      <c r="F8" s="47" t="str">
         <v>آزمایشی</v>
       </c>
     </row>
-    <row r="9" spans="1:6" s="50" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="72"/>
-      <c r="B9" s="72"/>
-      <c r="C9" s="72"/>
-      <c r="D9" s="72"/>
-      <c r="E9" s="72"/>
-      <c r="F9" s="72"/>
-    </row>
-    <row r="10" spans="1:6" s="50" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="72"/>
-      <c r="B10" s="72"/>
-      <c r="C10" s="72"/>
-      <c r="D10" s="72"/>
-      <c r="E10" s="72"/>
-      <c r="F10" s="72"/>
-    </row>
-    <row r="11" spans="1:6" s="50" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="72"/>
-      <c r="B11" s="72"/>
-      <c r="C11" s="72"/>
-      <c r="D11" s="72"/>
-      <c r="E11" s="72"/>
-      <c r="F11" s="72"/>
-    </row>
-    <row r="12" spans="1:6" s="50" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="72"/>
-      <c r="B12" s="72"/>
-      <c r="C12" s="72"/>
-      <c r="D12" s="72"/>
-      <c r="E12" s="72"/>
-      <c r="F12" s="72"/>
-    </row>
-    <row r="13" spans="1:6" s="50" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="72"/>
-      <c r="B13" s="72"/>
-      <c r="C13" s="72"/>
-      <c r="D13" s="72"/>
-      <c r="E13" s="72"/>
-      <c r="F13" s="72"/>
-    </row>
-    <row r="14" spans="1:6" s="50" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="72"/>
-      <c r="B14" s="72"/>
-      <c r="C14" s="72"/>
-      <c r="D14" s="72"/>
-      <c r="E14" s="72"/>
-      <c r="F14" s="72"/>
-    </row>
-    <row r="15" spans="1:6" s="50" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="72"/>
-      <c r="B15" s="72"/>
-      <c r="C15" s="72"/>
-      <c r="D15" s="72"/>
-      <c r="E15" s="72"/>
-      <c r="F15" s="72"/>
-    </row>
-    <row r="16" spans="1:6" s="50" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="72"/>
-      <c r="B16" s="72"/>
-      <c r="C16" s="72"/>
-      <c r="D16" s="72"/>
-      <c r="E16" s="72"/>
-      <c r="F16" s="72"/>
-    </row>
-    <row r="17" spans="1:6" s="50" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="72"/>
-      <c r="B17" s="72"/>
-      <c r="C17" s="72"/>
-      <c r="D17" s="72"/>
-      <c r="E17" s="72"/>
-      <c r="F17" s="72"/>
-    </row>
-    <row r="18" spans="1:6" s="50" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="72"/>
-      <c r="B18" s="72"/>
-      <c r="C18" s="72"/>
-      <c r="D18" s="72"/>
-      <c r="E18" s="72"/>
-      <c r="F18" s="72"/>
-    </row>
-    <row r="19" spans="1:6" s="50" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="72"/>
-      <c r="B19" s="72"/>
-      <c r="C19" s="72"/>
-      <c r="D19" s="72"/>
-      <c r="E19" s="72"/>
-      <c r="F19" s="72"/>
-    </row>
-    <row r="20" spans="1:6" s="50" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="72"/>
-      <c r="B20" s="72"/>
-      <c r="C20" s="72"/>
-      <c r="D20" s="72"/>
-      <c r="E20" s="72"/>
-      <c r="F20" s="72"/>
-    </row>
-    <row r="21" spans="1:6" s="50" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="72"/>
-      <c r="B21" s="72"/>
-      <c r="C21" s="72"/>
-      <c r="D21" s="72"/>
-      <c r="E21" s="72"/>
-      <c r="F21" s="72"/>
+    <row r="9" spans="1:6" s="36" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="47"/>
+      <c r="B9" s="47"/>
+      <c r="C9" s="47"/>
+      <c r="D9" s="47"/>
+      <c r="E9" s="47"/>
+      <c r="F9" s="47"/>
+    </row>
+    <row r="10" spans="1:6" s="36" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="47"/>
+      <c r="B10" s="47"/>
+      <c r="C10" s="47"/>
+      <c r="D10" s="47"/>
+      <c r="E10" s="47"/>
+      <c r="F10" s="47"/>
+    </row>
+    <row r="11" spans="1:6" s="36" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="47"/>
+      <c r="B11" s="47"/>
+      <c r="C11" s="47"/>
+      <c r="D11" s="47"/>
+      <c r="E11" s="47"/>
+      <c r="F11" s="47"/>
+    </row>
+    <row r="12" spans="1:6" s="36" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="47"/>
+      <c r="B12" s="47"/>
+      <c r="C12" s="47"/>
+      <c r="D12" s="47"/>
+      <c r="E12" s="47"/>
+      <c r="F12" s="47"/>
+    </row>
+    <row r="13" spans="1:6" s="36" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="47"/>
+      <c r="B13" s="47"/>
+      <c r="C13" s="47"/>
+      <c r="D13" s="47"/>
+      <c r="E13" s="47"/>
+      <c r="F13" s="47"/>
+    </row>
+    <row r="14" spans="1:6" s="36" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="47"/>
+      <c r="B14" s="47"/>
+      <c r="C14" s="47"/>
+      <c r="D14" s="47"/>
+      <c r="E14" s="47"/>
+      <c r="F14" s="47"/>
+    </row>
+    <row r="15" spans="1:6" s="36" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="47"/>
+      <c r="B15" s="47"/>
+      <c r="C15" s="47"/>
+      <c r="D15" s="47"/>
+      <c r="E15" s="47"/>
+      <c r="F15" s="47"/>
+    </row>
+    <row r="16" spans="1:6" s="36" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="47"/>
+      <c r="B16" s="47"/>
+      <c r="C16" s="47"/>
+      <c r="D16" s="47"/>
+      <c r="E16" s="47"/>
+      <c r="F16" s="47"/>
+    </row>
+    <row r="17" spans="1:6" s="36" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="47"/>
+      <c r="B17" s="47"/>
+      <c r="C17" s="47"/>
+      <c r="D17" s="47"/>
+      <c r="E17" s="47"/>
+      <c r="F17" s="47"/>
+    </row>
+    <row r="18" spans="1:6" s="36" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="47"/>
+      <c r="B18" s="47"/>
+      <c r="C18" s="47"/>
+      <c r="D18" s="47"/>
+      <c r="E18" s="47"/>
+      <c r="F18" s="47"/>
+    </row>
+    <row r="19" spans="1:6" s="36" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="47"/>
+      <c r="B19" s="47"/>
+      <c r="C19" s="47"/>
+      <c r="D19" s="47"/>
+      <c r="E19" s="47"/>
+      <c r="F19" s="47"/>
+    </row>
+    <row r="20" spans="1:6" s="36" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="47"/>
+      <c r="B20" s="47"/>
+      <c r="C20" s="47"/>
+      <c r="D20" s="47"/>
+      <c r="E20" s="47"/>
+      <c r="F20" s="47"/>
+    </row>
+    <row r="21" spans="1:6" s="36" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="47"/>
+      <c r="B21" s="47"/>
+      <c r="C21" s="47"/>
+      <c r="D21" s="47"/>
+      <c r="E21" s="47"/>
+      <c r="F21" s="47"/>
     </row>
     <row r="22" spans="1:6" ht="30.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
@@ -4693,56 +4586,56 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="26.25" x14ac:dyDescent="0.25">
-      <c r="A1" s="35" t="s">
+      <c r="A1" s="59" t="s">
         <v>19</v>
       </c>
-      <c r="B1" s="35"/>
-      <c r="C1" s="35"/>
-      <c r="D1" s="35"/>
-      <c r="E1" s="35"/>
-      <c r="G1" s="37" t="s">
+      <c r="B1" s="59"/>
+      <c r="C1" s="59"/>
+      <c r="D1" s="59"/>
+      <c r="E1" s="59"/>
+      <c r="G1" s="63" t="s">
         <v>19</v>
       </c>
-      <c r="H1" s="37"/>
-      <c r="I1" s="37"/>
-      <c r="J1" s="37"/>
-      <c r="K1" s="37"/>
-      <c r="L1" s="37"/>
+      <c r="H1" s="63"/>
+      <c r="I1" s="63"/>
+      <c r="J1" s="63"/>
+      <c r="K1" s="63"/>
+      <c r="L1" s="63"/>
     </row>
     <row r="2" spans="1:12" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="36" t="s">
+      <c r="A2" s="60" t="s">
         <v>111</v>
       </c>
-      <c r="B2" s="36"/>
-      <c r="C2" s="36"/>
-      <c r="D2" s="36"/>
-      <c r="E2" s="36"/>
-      <c r="G2" s="38" t="s">
+      <c r="B2" s="60"/>
+      <c r="C2" s="60"/>
+      <c r="D2" s="60"/>
+      <c r="E2" s="60"/>
+      <c r="G2" s="64" t="s">
         <v>111</v>
       </c>
-      <c r="H2" s="38"/>
-      <c r="I2" s="38"/>
-      <c r="J2" s="38"/>
-      <c r="K2" s="38"/>
-      <c r="L2" s="38"/>
+      <c r="H2" s="64"/>
+      <c r="I2" s="64"/>
+      <c r="J2" s="64"/>
+      <c r="K2" s="64"/>
+      <c r="L2" s="64"/>
     </row>
     <row r="3" spans="1:12" ht="20.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" spans="1:12" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A4" s="33" t="s">
+      <c r="A4" s="61" t="s">
         <v>112</v>
       </c>
-      <c r="B4" s="33"/>
-      <c r="C4" s="33"/>
-      <c r="D4" s="33"/>
-      <c r="E4" s="33"/>
-      <c r="G4" s="34" t="s">
+      <c r="B4" s="61"/>
+      <c r="C4" s="61"/>
+      <c r="D4" s="61"/>
+      <c r="E4" s="61"/>
+      <c r="G4" s="62" t="s">
         <v>123</v>
       </c>
-      <c r="H4" s="34"/>
-      <c r="I4" s="34"/>
-      <c r="J4" s="34"/>
-      <c r="K4" s="34"/>
-      <c r="L4" s="34"/>
+      <c r="H4" s="62"/>
+      <c r="I4" s="62"/>
+      <c r="J4" s="62"/>
+      <c r="K4" s="62"/>
+      <c r="L4" s="62"/>
     </row>
     <row r="5" spans="1:12" ht="19.5" x14ac:dyDescent="0.5">
       <c r="A5" s="21" t="s">
@@ -4757,16 +4650,16 @@
       <c r="D5" s="23" t="s">
         <v>116</v>
       </c>
-      <c r="G5" s="51" t="s">
+      <c r="G5" s="37" t="s">
         <v>124</v>
       </c>
-      <c r="H5" s="52" t="s">
+      <c r="H5" s="65" t="s">
         <v>57</v>
       </c>
-      <c r="I5" s="52"/>
-      <c r="J5" s="52"/>
-      <c r="K5" s="52"/>
-      <c r="L5" s="52"/>
+      <c r="I5" s="65"/>
+      <c r="J5" s="65"/>
+      <c r="K5" s="65"/>
+      <c r="L5" s="65"/>
     </row>
     <row r="6" spans="1:12" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
       <c r="A6" s="24">
@@ -4785,43 +4678,43 @@
         <f>COUNTIF(موجودی!J2:J1000,"تمام شده")</f>
         <v>11</v>
       </c>
-      <c r="G6" s="53" t="s">
+      <c r="G6" s="38" t="s">
         <v>2</v>
       </c>
-      <c r="H6" s="54" t="str">
+      <c r="H6" s="66" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(H5,موجودی!B:B,موجودی!A:A),"")</f>
         <v>K010</v>
       </c>
-      <c r="I6" s="54"/>
-      <c r="J6" s="54"/>
-      <c r="K6" s="54"/>
-      <c r="L6" s="54"/>
+      <c r="I6" s="66"/>
+      <c r="J6" s="66"/>
+      <c r="K6" s="66"/>
+      <c r="L6" s="66"/>
     </row>
     <row r="7" spans="1:12" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G7" s="59"/>
-      <c r="H7" s="58"/>
-      <c r="I7" s="58"/>
-      <c r="J7" s="58"/>
-      <c r="K7" s="58"/>
-      <c r="L7" s="62"/>
+      <c r="G7" s="40"/>
+      <c r="H7" s="39"/>
+      <c r="I7" s="39"/>
+      <c r="J7" s="39"/>
+      <c r="K7" s="39"/>
+      <c r="L7" s="43"/>
     </row>
     <row r="8" spans="1:12" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="34" t="s">
+      <c r="A8" s="62" t="s">
         <v>117</v>
       </c>
-      <c r="B8" s="34"/>
-      <c r="C8" s="34"/>
-      <c r="G8" s="60" t="s">
+      <c r="B8" s="62"/>
+      <c r="C8" s="62"/>
+      <c r="G8" s="41" t="s">
         <v>131</v>
       </c>
-      <c r="H8" s="56">
+      <c r="H8" s="48">
         <f>IFERROR(_xlfn.XLOOKUP(H6,'موجودی مبنا'!A:A,'موجودی مبنا'!D:D),0)</f>
         <v>44</v>
       </c>
-      <c r="I8" s="56"/>
-      <c r="J8" s="56"/>
-      <c r="K8" s="56"/>
-      <c r="L8" s="63"/>
+      <c r="I8" s="48"/>
+      <c r="J8" s="48"/>
+      <c r="K8" s="48"/>
+      <c r="L8" s="67"/>
     </row>
     <row r="9" spans="1:12" ht="19.5" x14ac:dyDescent="0.25">
       <c r="A9" s="21" t="s">
@@ -4833,32 +4726,32 @@
       <c r="C9" s="23" t="s">
         <v>118</v>
       </c>
-      <c r="G9" s="60" t="s">
+      <c r="G9" s="41" t="s">
         <v>15</v>
       </c>
-      <c r="H9" s="56">
+      <c r="H9" s="48">
         <f>SUMIF(tblvorood[کد کالا],H6,tblvorood[مقدار])</f>
-        <v>17</v>
-      </c>
-      <c r="I9" s="56"/>
-      <c r="J9" s="56"/>
-      <c r="K9" s="56"/>
-      <c r="L9" s="63"/>
+        <v>0</v>
+      </c>
+      <c r="I9" s="48"/>
+      <c r="J9" s="48"/>
+      <c r="K9" s="48"/>
+      <c r="L9" s="67"/>
     </row>
     <row r="10" spans="1:12" s="16" customFormat="1" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="30" t="str" cm="1">
         <f t="array" ref="A10">INDEX(tblvorood[شماره رسید],COUNTA(tblvorood[شماره رسید]))</f>
-        <v>R-050617-178</v>
+        <v>R-050617-173</v>
       </c>
       <c r="B10" s="31" t="str" cm="1">
         <f t="array" ref="B10">INDEX(tblvorood[تاریخ],COUNTA(tblvorood[تاریخ]))</f>
-        <v>1405/06/22</v>
+        <v>1405/06/17</v>
       </c>
       <c r="C10" s="32">
         <f>COUNTA(tblvorood[کد کالا])</f>
-        <v>4</v>
-      </c>
-      <c r="G10" s="61" t="s">
+        <v>2</v>
+      </c>
+      <c r="G10" s="42" t="s">
         <v>16</v>
       </c>
       <c r="H10" s="57">
@@ -4868,25 +4761,25 @@
       <c r="I10" s="57"/>
       <c r="J10" s="57"/>
       <c r="K10" s="57"/>
-      <c r="L10" s="64"/>
+      <c r="L10" s="69"/>
     </row>
     <row r="11" spans="1:12" s="16" customFormat="1" ht="40.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A11" s="33" t="s">
+      <c r="A11" s="61" t="s">
         <v>119</v>
       </c>
-      <c r="B11" s="33"/>
-      <c r="C11" s="33"/>
-      <c r="G11" s="61" t="s">
+      <c r="B11" s="61"/>
+      <c r="C11" s="61"/>
+      <c r="G11" s="42" t="s">
         <v>17</v>
       </c>
       <c r="H11" s="57">
         <f>H8+H9-H10</f>
-        <v>44</v>
+        <v>27</v>
       </c>
       <c r="I11" s="57"/>
       <c r="J11" s="57"/>
       <c r="K11" s="57"/>
-      <c r="L11" s="64"/>
+      <c r="L11" s="69"/>
     </row>
     <row r="12" spans="1:12" ht="19.5" x14ac:dyDescent="0.25">
       <c r="A12" s="21" t="s">
@@ -4908,103 +4801,103 @@
       <c r="C13" s="29"/>
     </row>
     <row r="14" spans="1:12" ht="40.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A14" s="33" t="s">
+      <c r="A14" s="61" t="s">
         <v>120</v>
       </c>
-      <c r="B14" s="33"/>
-      <c r="C14" s="33"/>
-      <c r="D14" s="33"/>
-      <c r="E14" s="33"/>
-      <c r="G14" s="33" t="s">
+      <c r="B14" s="61"/>
+      <c r="C14" s="61"/>
+      <c r="D14" s="61"/>
+      <c r="E14" s="61"/>
+      <c r="G14" s="61" t="s">
         <v>132</v>
       </c>
-      <c r="H14" s="33"/>
-      <c r="I14" s="33"/>
-      <c r="J14" s="33"/>
-      <c r="K14" s="33"/>
-      <c r="L14" s="33"/>
+      <c r="H14" s="61"/>
+      <c r="I14" s="61"/>
+      <c r="J14" s="61"/>
+      <c r="K14" s="61"/>
+      <c r="L14" s="61"/>
     </row>
     <row r="15" spans="1:12" ht="21" x14ac:dyDescent="0.25">
-      <c r="A15" s="48" t="s">
+      <c r="A15" s="34" t="s">
         <v>2</v>
       </c>
-      <c r="B15" s="48" t="s">
+      <c r="B15" s="34" t="s">
         <v>3</v>
       </c>
-      <c r="C15" s="48" t="s">
+      <c r="C15" s="34" t="s">
         <v>121</v>
       </c>
-      <c r="D15" s="48" t="s">
+      <c r="D15" s="34" t="s">
         <v>122</v>
       </c>
-      <c r="E15" s="48" t="s">
+      <c r="E15" s="34" t="s">
         <v>18</v>
       </c>
-      <c r="G15" s="46" t="s">
+      <c r="G15" s="33" t="s">
         <v>124</v>
       </c>
-      <c r="H15" s="47" t="s">
+      <c r="H15" s="68" t="s">
         <v>57</v>
       </c>
-      <c r="I15" s="47"/>
-      <c r="J15" s="47"/>
-      <c r="K15" s="47"/>
-      <c r="L15" s="47"/>
+      <c r="I15" s="68"/>
+      <c r="J15" s="68"/>
+      <c r="K15" s="68"/>
+      <c r="L15" s="68"/>
     </row>
     <row r="16" spans="1:12" ht="19.5" x14ac:dyDescent="0.25">
-      <c r="A16" s="50" t="str" cm="1">
+      <c r="A16" s="36" t="str" cm="1">
         <f t="array" ref="A16:E27">_xlfn._xlws.FILTER(_xlfn.CHOOSECOLS(موجودی!A2:J1000,1,2,8,9,10),(موجودی!J2:J1000="کم")+(موجودی!J2:J1000="تمام شده"),"")</f>
         <v>K001</v>
       </c>
-      <c r="B16" s="50" t="str">
+      <c r="B16" s="36" t="str">
         <v>استاد CW 75*3000</v>
       </c>
-      <c r="C16" s="50">
-        <v>0</v>
-      </c>
-      <c r="D16" s="50">
-        <v>0</v>
-      </c>
-      <c r="E16" s="50" t="str">
+      <c r="C16" s="36">
+        <v>0</v>
+      </c>
+      <c r="D16" s="36">
+        <v>0</v>
+      </c>
+      <c r="E16" s="36" t="str">
         <v>تمام شده</v>
       </c>
-      <c r="G16" s="48" t="s">
+      <c r="G16" s="34" t="s">
         <v>133</v>
       </c>
-      <c r="H16" s="48" t="s">
+      <c r="H16" s="34" t="s">
         <v>134</v>
       </c>
-      <c r="I16" s="48" t="s">
+      <c r="I16" s="34" t="s">
         <v>9</v>
       </c>
-      <c r="J16" s="48" t="s">
+      <c r="J16" s="34" t="s">
         <v>10</v>
       </c>
-      <c r="K16" s="48" t="s">
+      <c r="K16" s="34" t="s">
         <v>139</v>
       </c>
-      <c r="L16" s="48" t="s">
+      <c r="L16" s="34" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="17" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="50" t="str">
+      <c r="A17" s="36" t="str">
         <v>K002</v>
       </c>
-      <c r="B17" s="50" t="str">
+      <c r="B17" s="36" t="str">
         <v>استاد CW 100*3000</v>
       </c>
-      <c r="C17" s="50">
-        <v>0</v>
-      </c>
-      <c r="D17" s="50">
-        <v>0</v>
-      </c>
-      <c r="E17" s="50" t="str">
+      <c r="C17" s="36">
+        <v>0</v>
+      </c>
+      <c r="D17" s="36">
+        <v>0</v>
+      </c>
+      <c r="E17" s="36" t="str">
         <v>تمام شده</v>
       </c>
-      <c r="G17" s="65" t="str" cm="1">
-        <f t="array" ref="G17:L22">_xlfn.LET(
+      <c r="G17" s="45" t="str" cm="1">
+        <f t="array" ref="G17:L20">_xlfn.LET(
 _xlpm.کد,_xlfn.XLOOKUP($H$15,موجودی!B:B,موجودی!A:A),
 _xlpm.تاریخ_مبنا,_xlfn.XLOOKUP(_xlpm.کد,tblMabna[کد کالا],tblMabna[تاریخ مبنا]),
 _xlpm.مبنا,_xlfn._xlws.FILTER(
@@ -5066,350 +4959,314 @@
 )</f>
         <v>موجودی مبنا</v>
       </c>
-      <c r="H17" s="58" t="str">
+      <c r="H17" s="39" t="str">
         <v>-</v>
       </c>
-      <c r="I17" s="58" t="str">
+      <c r="I17" s="39" t="str">
         <v>1405/06/14</v>
       </c>
-      <c r="J17" s="58">
+      <c r="J17" s="39">
         <v>44</v>
       </c>
-      <c r="K17" s="58">
+      <c r="K17" s="39">
         <v>44</v>
       </c>
-      <c r="L17" s="62" t="str">
+      <c r="L17" s="43" t="str">
         <v>هر بسته 1000 عدد</v>
       </c>
     </row>
     <row r="18" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="50" t="str">
+      <c r="A18" s="36" t="str">
         <v>K003</v>
       </c>
-      <c r="B18" s="50" t="str">
+      <c r="B18" s="36" t="str">
         <v>استاد C 70*3500</v>
       </c>
-      <c r="C18" s="50">
-        <v>0</v>
-      </c>
-      <c r="D18" s="50">
-        <v>0</v>
-      </c>
-      <c r="E18" s="50" t="str">
+      <c r="C18" s="36">
+        <v>0</v>
+      </c>
+      <c r="D18" s="36">
+        <v>0</v>
+      </c>
+      <c r="E18" s="36" t="str">
         <v>تمام شده</v>
       </c>
-      <c r="G18" s="66" t="str">
+      <c r="G18" s="46" t="str">
         <v>خروج</v>
       </c>
-      <c r="H18" s="55" t="str">
+      <c r="H18" s="2" t="str">
         <v>H-050617-1</v>
       </c>
-      <c r="I18" s="55" t="str">
+      <c r="I18" s="2" t="str">
         <v>1405/06/17</v>
       </c>
-      <c r="J18" s="55">
+      <c r="J18" s="2">
         <v>2</v>
       </c>
-      <c r="K18" s="55">
+      <c r="K18" s="2">
         <v>42</v>
       </c>
-      <c r="L18" s="67" t="str">
+      <c r="L18" s="44" t="str">
         <v>خروج آزمایشی</v>
       </c>
     </row>
     <row r="19" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="50" t="str">
+      <c r="A19" s="36" t="str">
         <v>K004</v>
       </c>
-      <c r="B19" s="50" t="str">
+      <c r="B19" s="36" t="str">
         <v>رانر UW 70*4000</v>
       </c>
-      <c r="C19" s="50">
-        <v>0</v>
-      </c>
-      <c r="D19" s="50">
-        <v>0</v>
-      </c>
-      <c r="E19" s="50" t="str">
+      <c r="C19" s="36">
+        <v>0</v>
+      </c>
+      <c r="D19" s="36">
+        <v>0</v>
+      </c>
+      <c r="E19" s="36" t="str">
         <v>تمام شده</v>
       </c>
-      <c r="G19" s="66" t="str">
-        <v>ورود</v>
-      </c>
-      <c r="H19" s="55" t="str">
-        <v>R-050617-174</v>
-      </c>
-      <c r="I19" s="55" t="str">
+      <c r="G19" s="46" t="str">
+        <v>خروج</v>
+      </c>
+      <c r="H19" s="2" t="str">
+        <v>H-050617-2</v>
+      </c>
+      <c r="I19" s="2" t="str">
         <v>1405/06/18</v>
       </c>
-      <c r="J19" s="55">
-        <v>10</v>
-      </c>
-      <c r="K19" s="55">
-        <v>52</v>
-      </c>
-      <c r="L19" s="67" t="str">
-        <v>تستی</v>
+      <c r="J19" s="2">
+        <v>3</v>
+      </c>
+      <c r="K19" s="2">
+        <v>39</v>
+      </c>
+      <c r="L19" s="44" t="str">
+        <v>آزمایشی</v>
       </c>
     </row>
     <row r="20" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="50" t="str">
+      <c r="A20" s="36" t="str">
         <v>K005</v>
       </c>
-      <c r="B20" s="50" t="str">
+      <c r="B20" s="36" t="str">
         <v>رانر UW 75*4000</v>
       </c>
-      <c r="C20" s="50">
-        <v>0</v>
-      </c>
-      <c r="D20" s="50">
-        <v>0</v>
-      </c>
-      <c r="E20" s="50" t="str">
+      <c r="C20" s="36">
+        <v>0</v>
+      </c>
+      <c r="D20" s="36">
+        <v>0</v>
+      </c>
+      <c r="E20" s="36" t="str">
         <v>تمام شده</v>
       </c>
-      <c r="G20" s="66" t="str">
+      <c r="G20" s="46" t="str">
         <v>خروج</v>
       </c>
-      <c r="H20" s="55" t="str">
-        <v>H-050617-2</v>
-      </c>
-      <c r="I20" s="55" t="str">
-        <v>1405/06/18</v>
-      </c>
-      <c r="J20" s="55">
-        <v>3</v>
-      </c>
-      <c r="K20" s="55">
-        <v>49</v>
-      </c>
-      <c r="L20" s="67" t="str">
+      <c r="H20" s="2" t="str">
+        <v>H-050617-3</v>
+      </c>
+      <c r="I20" s="2" t="str">
+        <v>1405/06/19</v>
+      </c>
+      <c r="J20" s="2">
+        <v>12</v>
+      </c>
+      <c r="K20" s="2">
+        <v>27</v>
+      </c>
+      <c r="L20" s="44" t="str">
         <v>آزمایشی</v>
       </c>
     </row>
     <row r="21" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="50" t="str">
+      <c r="A21" s="36" t="str">
         <v>K006</v>
       </c>
-      <c r="B21" s="50" t="str">
+      <c r="B21" s="36" t="str">
         <v>رانر UW 100*4000</v>
       </c>
-      <c r="C21" s="50">
-        <v>0</v>
-      </c>
-      <c r="D21" s="50">
-        <v>0</v>
-      </c>
-      <c r="E21" s="50" t="str">
+      <c r="C21" s="36">
+        <v>0</v>
+      </c>
+      <c r="D21" s="36">
+        <v>0</v>
+      </c>
+      <c r="E21" s="36" t="str">
         <v>تمام شده</v>
       </c>
-      <c r="G21" s="66" t="str">
-        <v>خروج</v>
-      </c>
-      <c r="H21" s="55" t="str">
-        <v>H-050617-3</v>
-      </c>
-      <c r="I21" s="55" t="str">
-        <v>1405/06/19</v>
-      </c>
-      <c r="J21" s="55">
-        <v>12</v>
-      </c>
-      <c r="K21" s="55">
-        <v>37</v>
-      </c>
-      <c r="L21" s="67" t="str">
-        <v>آزمایشی</v>
-      </c>
+      <c r="G21" s="46"/>
+      <c r="L21" s="44"/>
     </row>
     <row r="22" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="50" t="str">
+      <c r="A22" s="36" t="str">
         <v>K007</v>
       </c>
-      <c r="B22" s="50" t="str">
+      <c r="B22" s="36" t="str">
         <v>پنل گچی 84 برگی MR_AK_H2</v>
       </c>
-      <c r="C22" s="50">
-        <v>0</v>
-      </c>
-      <c r="D22" s="50">
-        <v>0</v>
-      </c>
-      <c r="E22" s="50" t="str">
+      <c r="C22" s="36">
+        <v>0</v>
+      </c>
+      <c r="D22" s="36">
+        <v>0</v>
+      </c>
+      <c r="E22" s="36" t="str">
         <v>تمام شده</v>
       </c>
-      <c r="G22" s="66" t="str">
-        <v>ورود</v>
-      </c>
-      <c r="H22" s="55" t="str">
-        <v>R-050617-176</v>
-      </c>
-      <c r="I22" s="55" t="str">
-        <v>1405/06/20</v>
-      </c>
-      <c r="J22" s="55">
-        <v>7</v>
-      </c>
-      <c r="K22" s="55">
-        <v>44</v>
-      </c>
-      <c r="L22" s="67" t="str">
-        <v>آزمایشی</v>
-      </c>
+      <c r="G22" s="46"/>
+      <c r="L22" s="44"/>
     </row>
     <row r="23" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="50" t="str">
+      <c r="A23" s="36" t="str">
         <v>K008</v>
       </c>
-      <c r="B23" s="50" t="str">
+      <c r="B23" s="36" t="str">
         <v>پنل گچی 92 برگی RGPRO_AK</v>
       </c>
-      <c r="C23" s="50">
-        <v>0</v>
-      </c>
-      <c r="D23" s="50">
-        <v>0</v>
-      </c>
-      <c r="E23" s="50" t="str">
+      <c r="C23" s="36">
+        <v>0</v>
+      </c>
+      <c r="D23" s="36">
+        <v>0</v>
+      </c>
+      <c r="E23" s="36" t="str">
         <v>تمام شده</v>
       </c>
-      <c r="G23" s="66"/>
-      <c r="H23" s="55"/>
-      <c r="I23" s="55"/>
-      <c r="J23" s="55"/>
-      <c r="K23" s="55"/>
-      <c r="L23" s="67"/>
+      <c r="G23" s="46"/>
+      <c r="L23" s="44"/>
     </row>
     <row r="24" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="50" t="str">
+      <c r="A24" s="36" t="str">
         <v>K009</v>
       </c>
-      <c r="B24" s="50" t="str">
+      <c r="B24" s="36" t="str">
         <v>پنل گچی 100 برگی جی برد</v>
       </c>
-      <c r="C24" s="50">
-        <v>0</v>
-      </c>
-      <c r="D24" s="50">
-        <v>0</v>
-      </c>
-      <c r="E24" s="50" t="str">
+      <c r="C24" s="36">
+        <v>0</v>
+      </c>
+      <c r="D24" s="36">
+        <v>0</v>
+      </c>
+      <c r="E24" s="36" t="str">
         <v>تمام شده</v>
       </c>
     </row>
     <row r="25" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="50" t="str">
+      <c r="A25" s="36" t="str">
         <v>T006</v>
       </c>
-      <c r="B25" s="50" t="str">
+      <c r="B25" s="36" t="str">
         <v>الکترود 3/2 میکا</v>
       </c>
-      <c r="C25" s="50">
+      <c r="C25" s="36">
         <v>5</v>
       </c>
-      <c r="D25" s="50">
+      <c r="D25" s="36">
         <v>6</v>
       </c>
-      <c r="E25" s="50" t="str">
+      <c r="E25" s="36" t="str">
         <v>کم</v>
       </c>
     </row>
     <row r="26" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="50" t="str">
+      <c r="A26" s="36" t="str">
         <v>C001</v>
       </c>
-      <c r="B26" s="50" t="str">
+      <c r="B26" s="36" t="str">
         <v>ضد زنگ سناتور</v>
       </c>
-      <c r="C26" s="50">
-        <v>0</v>
-      </c>
-      <c r="D26" s="50">
-        <v>0</v>
-      </c>
-      <c r="E26" s="50" t="str">
+      <c r="C26" s="36">
+        <v>0</v>
+      </c>
+      <c r="D26" s="36">
+        <v>0</v>
+      </c>
+      <c r="E26" s="36" t="str">
         <v>تمام شده</v>
       </c>
     </row>
     <row r="27" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="50" t="str">
+      <c r="A27" s="36" t="str">
         <v>S001</v>
       </c>
-      <c r="B27" s="50" t="str">
+      <c r="B27" s="36" t="str">
         <v>قوطی 40*80</v>
       </c>
-      <c r="C27" s="50">
-        <v>0</v>
-      </c>
-      <c r="D27" s="50">
-        <v>0</v>
-      </c>
-      <c r="E27" s="50" t="str">
+      <c r="C27" s="36">
+        <v>0</v>
+      </c>
+      <c r="D27" s="36">
+        <v>0</v>
+      </c>
+      <c r="E27" s="36" t="str">
         <v>تمام شده</v>
       </c>
     </row>
     <row r="28" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="50"/>
-      <c r="B28" s="50"/>
-      <c r="C28" s="50"/>
-      <c r="D28" s="50"/>
-      <c r="E28" s="50"/>
+      <c r="A28" s="36"/>
+      <c r="B28" s="36"/>
+      <c r="C28" s="36"/>
+      <c r="D28" s="36"/>
+      <c r="E28" s="36"/>
     </row>
     <row r="29" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="50"/>
-      <c r="B29" s="50"/>
-      <c r="C29" s="50"/>
-      <c r="D29" s="50"/>
-      <c r="E29" s="50"/>
+      <c r="A29" s="36"/>
+      <c r="B29" s="36"/>
+      <c r="C29" s="36"/>
+      <c r="D29" s="36"/>
+      <c r="E29" s="36"/>
     </row>
     <row r="30" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="50"/>
-      <c r="B30" s="50"/>
-      <c r="C30" s="50"/>
-      <c r="D30" s="50"/>
-      <c r="E30" s="50"/>
+      <c r="A30" s="36"/>
+      <c r="B30" s="36"/>
+      <c r="C30" s="36"/>
+      <c r="D30" s="36"/>
+      <c r="E30" s="36"/>
     </row>
     <row r="31" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="50"/>
-      <c r="B31" s="50"/>
-      <c r="C31" s="50"/>
-      <c r="D31" s="50"/>
-      <c r="E31" s="50"/>
+      <c r="A31" s="36"/>
+      <c r="B31" s="36"/>
+      <c r="C31" s="36"/>
+      <c r="D31" s="36"/>
+      <c r="E31" s="36"/>
     </row>
     <row r="32" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="50"/>
-      <c r="B32" s="50"/>
-      <c r="C32" s="50"/>
-      <c r="D32" s="50"/>
-      <c r="E32" s="50"/>
+      <c r="A32" s="36"/>
+      <c r="B32" s="36"/>
+      <c r="C32" s="36"/>
+      <c r="D32" s="36"/>
+      <c r="E32" s="36"/>
     </row>
     <row r="33" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="50"/>
-      <c r="B33" s="50"/>
-      <c r="C33" s="50"/>
-      <c r="D33" s="50"/>
-      <c r="E33" s="50"/>
+      <c r="A33" s="36"/>
+      <c r="B33" s="36"/>
+      <c r="C33" s="36"/>
+      <c r="D33" s="36"/>
+      <c r="E33" s="36"/>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A34" s="50"/>
-      <c r="B34" s="50"/>
-      <c r="C34" s="50"/>
-      <c r="D34" s="50"/>
-      <c r="E34" s="50"/>
+      <c r="A34" s="36"/>
+      <c r="B34" s="36"/>
+      <c r="C34" s="36"/>
+      <c r="D34" s="36"/>
+      <c r="E34" s="36"/>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A35" s="50"/>
-      <c r="B35" s="50"/>
-      <c r="C35" s="50"/>
-      <c r="D35" s="50"/>
-      <c r="E35" s="50"/>
+      <c r="A35" s="36"/>
+      <c r="B35" s="36"/>
+      <c r="C35" s="36"/>
+      <c r="D35" s="36"/>
+      <c r="E35" s="36"/>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A36" s="50"/>
-      <c r="B36" s="50"/>
-      <c r="C36" s="50"/>
-      <c r="D36" s="50"/>
-      <c r="E36" s="50"/>
+      <c r="A36" s="36"/>
+      <c r="B36" s="36"/>
+      <c r="C36" s="36"/>
+      <c r="D36" s="36"/>
+      <c r="E36" s="36"/>
     </row>
   </sheetData>
   <mergeCells count="17">
@@ -5418,6 +5275,9 @@
     <mergeCell ref="A14:E14"/>
     <mergeCell ref="G4:L4"/>
     <mergeCell ref="G14:L14"/>
+    <mergeCell ref="H9:L9"/>
+    <mergeCell ref="H10:L10"/>
+    <mergeCell ref="H11:L11"/>
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A4:E4"/>
@@ -5427,9 +5287,6 @@
     <mergeCell ref="H5:L5"/>
     <mergeCell ref="H6:L6"/>
     <mergeCell ref="H8:L8"/>
-    <mergeCell ref="H9:L9"/>
-    <mergeCell ref="H10:L10"/>
-    <mergeCell ref="H11:L11"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>

</xml_diff>